<commit_message>
Replace em dashes, en dashes, and minus signs with plain hyphens
</commit_message>
<xml_diff>
--- a/outputs/variance_analysis.xlsx
+++ b/outputs/variance_analysis.xlsx
@@ -471,7 +471,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NorthPeak Analytics — FY2025 Budget vs. Actuals</t>
+          <t>NorthPeak Analytics - FY2025 Budget vs. Actuals</t>
         </is>
       </c>
     </row>
@@ -801,162 +801,162 @@
       </c>
       <c r="B1" s="8" t="inlineStr">
         <is>
-          <t>Revenue — Budget</t>
+          <t>Revenue - Budget</t>
         </is>
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>Revenue — Actual</t>
+          <t>Revenue - Actual</t>
         </is>
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Revenue — Var $</t>
+          <t>Revenue - Var $</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
         <is>
-          <t>Revenue — Var %</t>
+          <t>Revenue - Var %</t>
         </is>
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>COGS — Budget</t>
+          <t>COGS - Budget</t>
         </is>
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>COGS — Actual</t>
+          <t>COGS - Actual</t>
         </is>
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
-          <t>COGS — Var $</t>
+          <t>COGS - Var $</t>
         </is>
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
-          <t>COGS — Var %</t>
+          <t>COGS - Var %</t>
         </is>
       </c>
       <c r="J1" s="8" t="inlineStr">
         <is>
-          <t>Gross Profit — Budget</t>
+          <t>Gross Profit - Budget</t>
         </is>
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>Gross Profit — Actual</t>
+          <t>Gross Profit - Actual</t>
         </is>
       </c>
       <c r="L1" s="8" t="inlineStr">
         <is>
-          <t>Gross Profit — Var $</t>
+          <t>Gross Profit - Var $</t>
         </is>
       </c>
       <c r="M1" s="8" t="inlineStr">
         <is>
-          <t>Gross Profit — Var %</t>
+          <t>Gross Profit - Var %</t>
         </is>
       </c>
       <c r="N1" s="8" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing — Budget</t>
+          <t>Sales &amp; Marketing - Budget</t>
         </is>
       </c>
       <c r="O1" s="8" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing — Actual</t>
+          <t>Sales &amp; Marketing - Actual</t>
         </is>
       </c>
       <c r="P1" s="8" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing — Var $</t>
+          <t>Sales &amp; Marketing - Var $</t>
         </is>
       </c>
       <c r="Q1" s="8" t="inlineStr">
         <is>
-          <t>Sales &amp; Marketing — Var %</t>
+          <t>Sales &amp; Marketing - Var %</t>
         </is>
       </c>
       <c r="R1" s="8" t="inlineStr">
         <is>
-          <t>Research &amp; Development — Budget</t>
+          <t>Research &amp; Development - Budget</t>
         </is>
       </c>
       <c r="S1" s="8" t="inlineStr">
         <is>
-          <t>Research &amp; Development — Actual</t>
+          <t>Research &amp; Development - Actual</t>
         </is>
       </c>
       <c r="T1" s="8" t="inlineStr">
         <is>
-          <t>Research &amp; Development — Var $</t>
+          <t>Research &amp; Development - Var $</t>
         </is>
       </c>
       <c r="U1" s="8" t="inlineStr">
         <is>
-          <t>Research &amp; Development — Var %</t>
+          <t>Research &amp; Development - Var %</t>
         </is>
       </c>
       <c r="V1" s="8" t="inlineStr">
         <is>
-          <t>General &amp; Admin — Budget</t>
+          <t>General &amp; Admin - Budget</t>
         </is>
       </c>
       <c r="W1" s="8" t="inlineStr">
         <is>
-          <t>General &amp; Admin — Actual</t>
+          <t>General &amp; Admin - Actual</t>
         </is>
       </c>
       <c r="X1" s="8" t="inlineStr">
         <is>
-          <t>General &amp; Admin — Var $</t>
+          <t>General &amp; Admin - Var $</t>
         </is>
       </c>
       <c r="Y1" s="8" t="inlineStr">
         <is>
-          <t>General &amp; Admin — Var %</t>
+          <t>General &amp; Admin - Var %</t>
         </is>
       </c>
       <c r="Z1" s="8" t="inlineStr">
         <is>
-          <t>Total OpEx — Budget</t>
+          <t>Total OpEx - Budget</t>
         </is>
       </c>
       <c r="AA1" s="8" t="inlineStr">
         <is>
-          <t>Total OpEx — Actual</t>
+          <t>Total OpEx - Actual</t>
         </is>
       </c>
       <c r="AB1" s="8" t="inlineStr">
         <is>
-          <t>Total OpEx — Var $</t>
+          <t>Total OpEx - Var $</t>
         </is>
       </c>
       <c r="AC1" s="8" t="inlineStr">
         <is>
-          <t>Total OpEx — Var %</t>
+          <t>Total OpEx - Var %</t>
         </is>
       </c>
       <c r="AD1" s="8" t="inlineStr">
         <is>
-          <t>Operating Income — Budget</t>
+          <t>Operating Income - Budget</t>
         </is>
       </c>
       <c r="AE1" s="8" t="inlineStr">
         <is>
-          <t>Operating Income — Actual</t>
+          <t>Operating Income - Actual</t>
         </is>
       </c>
       <c r="AF1" s="8" t="inlineStr">
         <is>
-          <t>Operating Income — Var $</t>
+          <t>Operating Income - Var $</t>
         </is>
       </c>
       <c r="AG1" s="8" t="inlineStr">
         <is>
-          <t>Operating Income — Var %</t>
+          <t>Operating Income - Var %</t>
         </is>
       </c>
     </row>

</xml_diff>